<commit_message>
Updated: rerun analysis, documents rewritten, metadata stripped, preparing to anonymize
</commit_message>
<xml_diff>
--- a/documents/results_raw_two_seeds.xlsx
+++ b/documents/results_raw_two_seeds.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Nagc2/Desktop/so101-vla-data-study/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8886E8A8-9152-BE4C-B57A-D7EE11FBD221}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0806E5B7-DF43-8543-BE96-F730C923154C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="21460" xr2:uid="{E9882473-D8D3-4249-9541-943B7997CA3D}"/>
+    <workbookView xWindow="-20" yWindow="700" windowWidth="17120" windowHeight="20200" xr2:uid="{E9882473-D8D3-4249-9541-943B7997CA3D}"/>
   </bookViews>
   <sheets>
     <sheet name="results" sheetId="1" r:id="rId1"/>
@@ -2934,7 +2934,7 @@
         <v>0</v>
       </c>
       <c r="H78" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I78" t="s">
         <v>85</v>
@@ -2986,7 +2986,7 @@
         <v>0</v>
       </c>
       <c r="H80" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I80" t="s">
         <v>85</v>
@@ -3064,7 +3064,7 @@
         <v>0</v>
       </c>
       <c r="H83" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I83" t="s">
         <v>85</v>
@@ -3142,7 +3142,7 @@
         <v>0</v>
       </c>
       <c r="H86" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I86" t="s">
         <v>85</v>
@@ -3999,7 +3999,7 @@
         <v>0</v>
       </c>
       <c r="H117" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I117" t="s">
         <v>85</v>
@@ -4320,7 +4320,7 @@
         <v>0</v>
       </c>
       <c r="H129" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I129" t="s">
         <v>85</v>
@@ -4693,7 +4693,7 @@
         <v>0</v>
       </c>
       <c r="H143" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I143" t="s">
         <v>85</v>

</xml_diff>

<commit_message>
Added density probe experiment, updated files and results
</commit_message>
<xml_diff>
--- a/documents/results_raw_two_seeds.xlsx
+++ b/documents/results_raw_two_seeds.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Nagc2/Desktop/so101-vla-data-study/documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0806E5B7-DF43-8543-BE96-F730C923154C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5A8A0BD-A0C8-B14A-ACF5-5F8762CCFB7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="700" windowWidth="17120" windowHeight="20200" xr2:uid="{E9882473-D8D3-4249-9541-943B7997CA3D}"/>
+    <workbookView xWindow="-20" yWindow="680" windowWidth="17120" windowHeight="20180" activeTab="1" xr2:uid="{E9882473-D8D3-4249-9541-943B7997CA3D}"/>
   </bookViews>
   <sheets>
     <sheet name="results" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -66,7 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3503" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3743" uniqueCount="144">
   <si>
     <t>condition</t>
   </si>
@@ -478,12 +478,33 @@
   <si>
     <t>went to t6, bumped cube at last second</t>
   </si>
+  <si>
+    <t>density</t>
+  </si>
+  <si>
+    <t>trained_t2</t>
+  </si>
+  <si>
+    <t>went at t2</t>
+  </si>
+  <si>
+    <t>went towards T6, a bit to the left as if near the cube, shifted lefts slightly but didn't make it down to the cube</t>
+  </si>
+  <si>
+    <t>went to t2, started shifting very slightly to right but stayed by T2</t>
+  </si>
+  <si>
+    <t>went to t6 at first, then to the middle and stayed there hovering, and then to t2</t>
+  </si>
+  <si>
+    <t>went to T6, then towards the middle a bit but stayed facing T6</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -495,6 +516,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -16992,8 +17019,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70ED3EF9-8438-1949-8DDB-D638E98A674E}">
-  <dimension ref="A1:K63"/>
+  <dimension ref="A1:K108"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="16" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -18705,7 +18735,1223 @@
         <v>136</v>
       </c>
     </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>137</v>
+      </c>
+      <c r="B64" t="s">
+        <v>3</v>
+      </c>
+      <c r="C64">
+        <v>1000</v>
+      </c>
+      <c r="D64">
+        <v>1</v>
+      </c>
+      <c r="E64" t="s">
+        <v>35</v>
+      </c>
+      <c r="F64">
+        <v>1</v>
+      </c>
+      <c r="H64" t="s">
+        <v>13</v>
+      </c>
+      <c r="I64" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>137</v>
+      </c>
+      <c r="B65" t="s">
+        <v>3</v>
+      </c>
+      <c r="C65">
+        <v>1000</v>
+      </c>
+      <c r="D65">
+        <v>2</v>
+      </c>
+      <c r="E65" t="s">
+        <v>35</v>
+      </c>
+      <c r="F65">
+        <v>1</v>
+      </c>
+      <c r="H65" t="s">
+        <v>13</v>
+      </c>
+      <c r="I65" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>137</v>
+      </c>
+      <c r="B66" t="s">
+        <v>3</v>
+      </c>
+      <c r="C66">
+        <v>1000</v>
+      </c>
+      <c r="D66">
+        <v>3</v>
+      </c>
+      <c r="E66" t="s">
+        <v>35</v>
+      </c>
+      <c r="F66">
+        <v>1</v>
+      </c>
+      <c r="H66" t="s">
+        <v>13</v>
+      </c>
+      <c r="I66" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>137</v>
+      </c>
+      <c r="B67" t="s">
+        <v>3</v>
+      </c>
+      <c r="C67">
+        <v>1000</v>
+      </c>
+      <c r="D67">
+        <v>4</v>
+      </c>
+      <c r="E67" t="s">
+        <v>35</v>
+      </c>
+      <c r="F67">
+        <v>1</v>
+      </c>
+      <c r="H67" t="s">
+        <v>13</v>
+      </c>
+      <c r="I67" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>137</v>
+      </c>
+      <c r="B68" t="s">
+        <v>3</v>
+      </c>
+      <c r="C68">
+        <v>1000</v>
+      </c>
+      <c r="D68">
+        <v>5</v>
+      </c>
+      <c r="E68" t="s">
+        <v>35</v>
+      </c>
+      <c r="F68">
+        <v>1</v>
+      </c>
+      <c r="H68" t="s">
+        <v>13</v>
+      </c>
+      <c r="I68" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>137</v>
+      </c>
+      <c r="B69" t="s">
+        <v>3</v>
+      </c>
+      <c r="C69">
+        <v>1000</v>
+      </c>
+      <c r="D69">
+        <v>6</v>
+      </c>
+      <c r="E69" t="s">
+        <v>35</v>
+      </c>
+      <c r="F69">
+        <v>1</v>
+      </c>
+      <c r="H69" t="s">
+        <v>13</v>
+      </c>
+      <c r="I69" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>137</v>
+      </c>
+      <c r="B70" t="s">
+        <v>3</v>
+      </c>
+      <c r="C70">
+        <v>1000</v>
+      </c>
+      <c r="D70">
+        <v>7</v>
+      </c>
+      <c r="E70" t="s">
+        <v>35</v>
+      </c>
+      <c r="F70">
+        <v>1</v>
+      </c>
+      <c r="H70" t="s">
+        <v>13</v>
+      </c>
+      <c r="I70" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>137</v>
+      </c>
+      <c r="B71" t="s">
+        <v>3</v>
+      </c>
+      <c r="C71">
+        <v>1000</v>
+      </c>
+      <c r="D71">
+        <v>8</v>
+      </c>
+      <c r="E71" t="s">
+        <v>35</v>
+      </c>
+      <c r="F71">
+        <v>1</v>
+      </c>
+      <c r="H71" t="s">
+        <v>13</v>
+      </c>
+      <c r="I71" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>137</v>
+      </c>
+      <c r="B72" t="s">
+        <v>3</v>
+      </c>
+      <c r="C72">
+        <v>1000</v>
+      </c>
+      <c r="D72">
+        <v>9</v>
+      </c>
+      <c r="E72" t="s">
+        <v>35</v>
+      </c>
+      <c r="F72">
+        <v>1</v>
+      </c>
+      <c r="H72" t="s">
+        <v>13</v>
+      </c>
+      <c r="I72" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>137</v>
+      </c>
+      <c r="B73" t="s">
+        <v>3</v>
+      </c>
+      <c r="C73">
+        <v>1000</v>
+      </c>
+      <c r="D73">
+        <v>10</v>
+      </c>
+      <c r="E73" t="s">
+        <v>35</v>
+      </c>
+      <c r="F73">
+        <v>1</v>
+      </c>
+      <c r="H73" t="s">
+        <v>13</v>
+      </c>
+      <c r="I73" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>137</v>
+      </c>
+      <c r="B74" t="s">
+        <v>3</v>
+      </c>
+      <c r="C74">
+        <v>1000</v>
+      </c>
+      <c r="D74">
+        <v>11</v>
+      </c>
+      <c r="E74" t="s">
+        <v>35</v>
+      </c>
+      <c r="F74">
+        <v>1</v>
+      </c>
+      <c r="H74" t="s">
+        <v>13</v>
+      </c>
+      <c r="I74" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>137</v>
+      </c>
+      <c r="B75" t="s">
+        <v>3</v>
+      </c>
+      <c r="C75">
+        <v>1000</v>
+      </c>
+      <c r="D75">
+        <v>12</v>
+      </c>
+      <c r="E75" t="s">
+        <v>35</v>
+      </c>
+      <c r="F75">
+        <v>1</v>
+      </c>
+      <c r="H75" t="s">
+        <v>13</v>
+      </c>
+      <c r="I75" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>137</v>
+      </c>
+      <c r="B76" t="s">
+        <v>3</v>
+      </c>
+      <c r="C76">
+        <v>1000</v>
+      </c>
+      <c r="D76">
+        <v>13</v>
+      </c>
+      <c r="E76" t="s">
+        <v>35</v>
+      </c>
+      <c r="F76">
+        <v>1</v>
+      </c>
+      <c r="H76" t="s">
+        <v>13</v>
+      </c>
+      <c r="I76" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>137</v>
+      </c>
+      <c r="B77" t="s">
+        <v>3</v>
+      </c>
+      <c r="C77">
+        <v>1000</v>
+      </c>
+      <c r="D77">
+        <v>14</v>
+      </c>
+      <c r="E77" t="s">
+        <v>35</v>
+      </c>
+      <c r="F77">
+        <v>1</v>
+      </c>
+      <c r="H77" t="s">
+        <v>13</v>
+      </c>
+      <c r="I77" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>137</v>
+      </c>
+      <c r="B78" t="s">
+        <v>3</v>
+      </c>
+      <c r="C78">
+        <v>1000</v>
+      </c>
+      <c r="D78">
+        <v>15</v>
+      </c>
+      <c r="E78" t="s">
+        <v>35</v>
+      </c>
+      <c r="F78">
+        <v>1</v>
+      </c>
+      <c r="H78" t="s">
+        <v>13</v>
+      </c>
+      <c r="I78" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>137</v>
+      </c>
+      <c r="B79" t="s">
+        <v>138</v>
+      </c>
+      <c r="C79">
+        <v>1000</v>
+      </c>
+      <c r="D79">
+        <v>1</v>
+      </c>
+      <c r="E79" t="s">
+        <v>35</v>
+      </c>
+      <c r="F79">
+        <v>1</v>
+      </c>
+      <c r="H79" t="s">
+        <v>13</v>
+      </c>
+      <c r="I79" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>137</v>
+      </c>
+      <c r="B80" t="s">
+        <v>138</v>
+      </c>
+      <c r="C80">
+        <v>1000</v>
+      </c>
+      <c r="D80">
+        <v>2</v>
+      </c>
+      <c r="E80" t="s">
+        <v>35</v>
+      </c>
+      <c r="F80">
+        <v>1</v>
+      </c>
+      <c r="H80" t="s">
+        <v>13</v>
+      </c>
+      <c r="I80" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>137</v>
+      </c>
+      <c r="B81" t="s">
+        <v>138</v>
+      </c>
+      <c r="C81">
+        <v>1000</v>
+      </c>
+      <c r="D81">
+        <v>3</v>
+      </c>
+      <c r="E81" t="s">
+        <v>35</v>
+      </c>
+      <c r="F81">
+        <v>1</v>
+      </c>
+      <c r="H81" t="s">
+        <v>13</v>
+      </c>
+      <c r="I81" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>137</v>
+      </c>
+      <c r="B82" t="s">
+        <v>138</v>
+      </c>
+      <c r="C82">
+        <v>1000</v>
+      </c>
+      <c r="D82">
+        <v>4</v>
+      </c>
+      <c r="E82" t="s">
+        <v>35</v>
+      </c>
+      <c r="F82">
+        <v>1</v>
+      </c>
+      <c r="H82" t="s">
+        <v>13</v>
+      </c>
+      <c r="I82" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>137</v>
+      </c>
+      <c r="B83" t="s">
+        <v>138</v>
+      </c>
+      <c r="C83">
+        <v>1000</v>
+      </c>
+      <c r="D83">
+        <v>5</v>
+      </c>
+      <c r="E83" t="s">
+        <v>35</v>
+      </c>
+      <c r="F83">
+        <v>1</v>
+      </c>
+      <c r="H83" t="s">
+        <v>13</v>
+      </c>
+      <c r="I83" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>137</v>
+      </c>
+      <c r="B84" t="s">
+        <v>138</v>
+      </c>
+      <c r="C84">
+        <v>1000</v>
+      </c>
+      <c r="D84">
+        <v>6</v>
+      </c>
+      <c r="E84" t="s">
+        <v>35</v>
+      </c>
+      <c r="F84">
+        <v>1</v>
+      </c>
+      <c r="H84" t="s">
+        <v>13</v>
+      </c>
+      <c r="I84" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>137</v>
+      </c>
+      <c r="B85" t="s">
+        <v>138</v>
+      </c>
+      <c r="C85">
+        <v>1000</v>
+      </c>
+      <c r="D85">
+        <v>7</v>
+      </c>
+      <c r="E85" t="s">
+        <v>35</v>
+      </c>
+      <c r="F85">
+        <v>1</v>
+      </c>
+      <c r="H85" t="s">
+        <v>13</v>
+      </c>
+      <c r="I85" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>137</v>
+      </c>
+      <c r="B86" t="s">
+        <v>138</v>
+      </c>
+      <c r="C86">
+        <v>1000</v>
+      </c>
+      <c r="D86">
+        <v>8</v>
+      </c>
+      <c r="E86" t="s">
+        <v>35</v>
+      </c>
+      <c r="F86">
+        <v>1</v>
+      </c>
+      <c r="H86" t="s">
+        <v>13</v>
+      </c>
+      <c r="I86" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>137</v>
+      </c>
+      <c r="B87" t="s">
+        <v>138</v>
+      </c>
+      <c r="C87">
+        <v>1000</v>
+      </c>
+      <c r="D87">
+        <v>9</v>
+      </c>
+      <c r="E87" t="s">
+        <v>35</v>
+      </c>
+      <c r="F87">
+        <v>1</v>
+      </c>
+      <c r="H87" t="s">
+        <v>13</v>
+      </c>
+      <c r="I87" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>137</v>
+      </c>
+      <c r="B88" t="s">
+        <v>138</v>
+      </c>
+      <c r="C88">
+        <v>1000</v>
+      </c>
+      <c r="D88">
+        <v>10</v>
+      </c>
+      <c r="E88" t="s">
+        <v>35</v>
+      </c>
+      <c r="F88">
+        <v>1</v>
+      </c>
+      <c r="H88" t="s">
+        <v>13</v>
+      </c>
+      <c r="I88" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>137</v>
+      </c>
+      <c r="B89" t="s">
+        <v>138</v>
+      </c>
+      <c r="C89">
+        <v>1000</v>
+      </c>
+      <c r="D89">
+        <v>11</v>
+      </c>
+      <c r="E89" t="s">
+        <v>35</v>
+      </c>
+      <c r="F89">
+        <v>1</v>
+      </c>
+      <c r="H89" t="s">
+        <v>13</v>
+      </c>
+      <c r="I89" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>137</v>
+      </c>
+      <c r="B90" t="s">
+        <v>138</v>
+      </c>
+      <c r="C90">
+        <v>1000</v>
+      </c>
+      <c r="D90">
+        <v>12</v>
+      </c>
+      <c r="E90" t="s">
+        <v>35</v>
+      </c>
+      <c r="F90">
+        <v>1</v>
+      </c>
+      <c r="H90" t="s">
+        <v>13</v>
+      </c>
+      <c r="I90" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>137</v>
+      </c>
+      <c r="B91" t="s">
+        <v>138</v>
+      </c>
+      <c r="C91">
+        <v>1000</v>
+      </c>
+      <c r="D91">
+        <v>13</v>
+      </c>
+      <c r="E91" t="s">
+        <v>35</v>
+      </c>
+      <c r="F91">
+        <v>1</v>
+      </c>
+      <c r="H91" t="s">
+        <v>13</v>
+      </c>
+      <c r="I91" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>137</v>
+      </c>
+      <c r="B92" t="s">
+        <v>138</v>
+      </c>
+      <c r="C92">
+        <v>1000</v>
+      </c>
+      <c r="D92">
+        <v>14</v>
+      </c>
+      <c r="E92" t="s">
+        <v>35</v>
+      </c>
+      <c r="F92">
+        <v>1</v>
+      </c>
+      <c r="H92" t="s">
+        <v>13</v>
+      </c>
+      <c r="I92" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>137</v>
+      </c>
+      <c r="B93" t="s">
+        <v>138</v>
+      </c>
+      <c r="C93">
+        <v>1000</v>
+      </c>
+      <c r="D93">
+        <v>15</v>
+      </c>
+      <c r="E93" t="s">
+        <v>35</v>
+      </c>
+      <c r="F93">
+        <v>1</v>
+      </c>
+      <c r="H93" t="s">
+        <v>13</v>
+      </c>
+      <c r="I93" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>137</v>
+      </c>
+      <c r="B94" t="s">
+        <v>4</v>
+      </c>
+      <c r="C94">
+        <v>1000</v>
+      </c>
+      <c r="D94">
+        <v>1</v>
+      </c>
+      <c r="E94" t="s">
+        <v>23</v>
+      </c>
+      <c r="F94">
+        <v>0</v>
+      </c>
+      <c r="H94" t="s">
+        <v>62</v>
+      </c>
+      <c r="I94" t="s">
+        <v>85</v>
+      </c>
+      <c r="K94" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>137</v>
+      </c>
+      <c r="B95" t="s">
+        <v>4</v>
+      </c>
+      <c r="C95">
+        <v>1000</v>
+      </c>
+      <c r="D95">
+        <v>2</v>
+      </c>
+      <c r="E95" t="s">
+        <v>23</v>
+      </c>
+      <c r="F95">
+        <v>0</v>
+      </c>
+      <c r="H95" t="s">
+        <v>62</v>
+      </c>
+      <c r="I95" t="s">
+        <v>85</v>
+      </c>
+      <c r="K95" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>137</v>
+      </c>
+      <c r="B96" t="s">
+        <v>4</v>
+      </c>
+      <c r="C96">
+        <v>1000</v>
+      </c>
+      <c r="D96">
+        <v>3</v>
+      </c>
+      <c r="E96" t="s">
+        <v>23</v>
+      </c>
+      <c r="F96">
+        <v>0</v>
+      </c>
+      <c r="H96" t="s">
+        <v>62</v>
+      </c>
+      <c r="I96" t="s">
+        <v>85</v>
+      </c>
+      <c r="K96" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>137</v>
+      </c>
+      <c r="B97" t="s">
+        <v>4</v>
+      </c>
+      <c r="C97">
+        <v>1000</v>
+      </c>
+      <c r="D97">
+        <v>4</v>
+      </c>
+      <c r="E97" t="s">
+        <v>24</v>
+      </c>
+      <c r="F97">
+        <v>0</v>
+      </c>
+      <c r="H97" t="s">
+        <v>62</v>
+      </c>
+      <c r="I97" t="s">
+        <v>85</v>
+      </c>
+      <c r="K97" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>137</v>
+      </c>
+      <c r="B98" t="s">
+        <v>4</v>
+      </c>
+      <c r="C98">
+        <v>1000</v>
+      </c>
+      <c r="D98">
+        <v>5</v>
+      </c>
+      <c r="E98" t="s">
+        <v>24</v>
+      </c>
+      <c r="F98">
+        <v>0</v>
+      </c>
+      <c r="H98" t="s">
+        <v>62</v>
+      </c>
+      <c r="I98" t="s">
+        <v>85</v>
+      </c>
+      <c r="K98" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>137</v>
+      </c>
+      <c r="B99" t="s">
+        <v>4</v>
+      </c>
+      <c r="C99">
+        <v>1000</v>
+      </c>
+      <c r="D99">
+        <v>6</v>
+      </c>
+      <c r="E99" t="s">
+        <v>24</v>
+      </c>
+      <c r="F99">
+        <v>0</v>
+      </c>
+      <c r="H99" t="s">
+        <v>62</v>
+      </c>
+      <c r="I99" t="s">
+        <v>85</v>
+      </c>
+      <c r="K99" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>137</v>
+      </c>
+      <c r="B100" t="s">
+        <v>4</v>
+      </c>
+      <c r="C100">
+        <v>1000</v>
+      </c>
+      <c r="D100">
+        <v>7</v>
+      </c>
+      <c r="E100" t="s">
+        <v>25</v>
+      </c>
+      <c r="F100">
+        <v>0</v>
+      </c>
+      <c r="H100" t="s">
+        <v>62</v>
+      </c>
+      <c r="I100" t="s">
+        <v>85</v>
+      </c>
+      <c r="K100" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>137</v>
+      </c>
+      <c r="B101" t="s">
+        <v>4</v>
+      </c>
+      <c r="C101">
+        <v>1000</v>
+      </c>
+      <c r="D101">
+        <v>8</v>
+      </c>
+      <c r="E101" t="s">
+        <v>25</v>
+      </c>
+      <c r="F101">
+        <v>0</v>
+      </c>
+      <c r="H101" t="s">
+        <v>62</v>
+      </c>
+      <c r="I101" t="s">
+        <v>85</v>
+      </c>
+      <c r="K101" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>137</v>
+      </c>
+      <c r="B102" t="s">
+        <v>4</v>
+      </c>
+      <c r="C102">
+        <v>1000</v>
+      </c>
+      <c r="D102">
+        <v>9</v>
+      </c>
+      <c r="E102" t="s">
+        <v>25</v>
+      </c>
+      <c r="F102">
+        <v>0</v>
+      </c>
+      <c r="H102" t="s">
+        <v>62</v>
+      </c>
+      <c r="I102" t="s">
+        <v>85</v>
+      </c>
+      <c r="K102" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>137</v>
+      </c>
+      <c r="B103" t="s">
+        <v>4</v>
+      </c>
+      <c r="C103">
+        <v>1000</v>
+      </c>
+      <c r="D103">
+        <v>10</v>
+      </c>
+      <c r="E103" t="s">
+        <v>26</v>
+      </c>
+      <c r="F103">
+        <v>0</v>
+      </c>
+      <c r="H103" t="s">
+        <v>62</v>
+      </c>
+      <c r="I103" t="s">
+        <v>85</v>
+      </c>
+      <c r="K103" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>137</v>
+      </c>
+      <c r="B104" t="s">
+        <v>4</v>
+      </c>
+      <c r="C104">
+        <v>1000</v>
+      </c>
+      <c r="D104">
+        <v>11</v>
+      </c>
+      <c r="E104" t="s">
+        <v>26</v>
+      </c>
+      <c r="F104">
+        <v>0</v>
+      </c>
+      <c r="H104" t="s">
+        <v>62</v>
+      </c>
+      <c r="I104" t="s">
+        <v>85</v>
+      </c>
+      <c r="K104" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>137</v>
+      </c>
+      <c r="B105" t="s">
+        <v>4</v>
+      </c>
+      <c r="C105">
+        <v>1000</v>
+      </c>
+      <c r="D105">
+        <v>12</v>
+      </c>
+      <c r="E105" t="s">
+        <v>26</v>
+      </c>
+      <c r="F105">
+        <v>0</v>
+      </c>
+      <c r="H105" t="s">
+        <v>62</v>
+      </c>
+      <c r="I105" t="s">
+        <v>85</v>
+      </c>
+      <c r="K105" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
+        <v>137</v>
+      </c>
+      <c r="B106" t="s">
+        <v>4</v>
+      </c>
+      <c r="C106">
+        <v>1000</v>
+      </c>
+      <c r="D106">
+        <v>13</v>
+      </c>
+      <c r="E106" t="s">
+        <v>27</v>
+      </c>
+      <c r="F106">
+        <v>0</v>
+      </c>
+      <c r="H106" t="s">
+        <v>62</v>
+      </c>
+      <c r="I106" t="s">
+        <v>85</v>
+      </c>
+      <c r="K106" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>137</v>
+      </c>
+      <c r="B107" t="s">
+        <v>4</v>
+      </c>
+      <c r="C107">
+        <v>1000</v>
+      </c>
+      <c r="D107">
+        <v>14</v>
+      </c>
+      <c r="E107" t="s">
+        <v>27</v>
+      </c>
+      <c r="F107">
+        <v>0</v>
+      </c>
+      <c r="H107" t="s">
+        <v>62</v>
+      </c>
+      <c r="I107" t="s">
+        <v>85</v>
+      </c>
+      <c r="K107" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>137</v>
+      </c>
+      <c r="B108" t="s">
+        <v>4</v>
+      </c>
+      <c r="C108">
+        <v>1000</v>
+      </c>
+      <c r="D108">
+        <v>15</v>
+      </c>
+      <c r="E108" t="s">
+        <v>27</v>
+      </c>
+      <c r="F108">
+        <v>0</v>
+      </c>
+      <c r="H108" t="s">
+        <v>62</v>
+      </c>
+      <c r="I108" t="s">
+        <v>85</v>
+      </c>
+      <c r="K108" t="s">
+        <v>143</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I30" xr:uid="{18A8A8D7-FBDA-3C4C-ABC9-DBF5BA7B7A8A}">
       <formula1>"None, Failed, Succeeded"</formula1>

</xml_diff>